<commit_message>
git Commit "Stock Quantity and Media Library"
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/zltUI/ZltTestData.xlsx
+++ b/src/test/resources/testdata/zltUI/ZltTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sarojkumar\git\ZlaataQAsever36\src\test\resources\testdata\zltUI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\git\ZlaataQAsever\Ref\src\test\resources\testdata\zltUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B14D6B7-D4B2-4272-ABC4-BD75FD510A3F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64AC72B-81E6-4734-80FF-846547B1781F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{905F911F-FA1A-4DDD-B945-7467E9458D34}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9507" uniqueCount="993">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9592" uniqueCount="1000">
   <si>
     <t>S.No</t>
   </si>
@@ -3005,6 +3005,27 @@
   </si>
   <si>
     <t>Verify New Label functionality in user app.</t>
+  </si>
+  <si>
+    <t>Media Library</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_ML_01</t>
+  </si>
+  <si>
+    <t>Verify adding a new image to the product in Media Library and checking in UI</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_ML_01</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_ML_02</t>
+  </si>
+  <si>
+    <t>Verify that changing the brand type in Media Library is reflected on the product page</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_ML_02</t>
   </si>
 </sst>
 </file>
@@ -3647,6 +3668,24 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3673,24 +3712,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4494,7 +4515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75D1F84-2AD1-4552-9C1F-85B59D75CCFA}">
-  <dimension ref="A1:Z290"/>
+  <dimension ref="A1:Z293"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -5245,18 +5266,18 @@
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="95" t="s">
+      <c r="A24" s="86" t="s">
         <v>156</v>
       </c>
-      <c r="B24" s="96"/>
-      <c r="C24" s="96"/>
-      <c r="D24" s="96"/>
-      <c r="E24" s="96"/>
-      <c r="F24" s="96"/>
-      <c r="G24" s="96"/>
-      <c r="H24" s="96"/>
-      <c r="I24" s="96"/>
-      <c r="J24" s="97"/>
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="87"/>
+      <c r="G24" s="87"/>
+      <c r="H24" s="87"/>
+      <c r="I24" s="87"/>
+      <c r="J24" s="88"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="18">
@@ -5643,18 +5664,18 @@
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="98" t="s">
+      <c r="A37" s="89" t="s">
         <v>172</v>
       </c>
-      <c r="B37" s="99"/>
-      <c r="C37" s="99"/>
-      <c r="D37" s="99"/>
-      <c r="E37" s="99"/>
-      <c r="F37" s="99"/>
-      <c r="G37" s="99"/>
-      <c r="H37" s="99"/>
-      <c r="I37" s="99"/>
-      <c r="J37" s="100"/>
+      <c r="B37" s="90"/>
+      <c r="C37" s="90"/>
+      <c r="D37" s="90"/>
+      <c r="E37" s="90"/>
+      <c r="F37" s="90"/>
+      <c r="G37" s="90"/>
+      <c r="H37" s="90"/>
+      <c r="I37" s="90"/>
+      <c r="J37" s="91"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="10">
@@ -6201,18 +6222,18 @@
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A55" s="98" t="s">
+      <c r="A55" s="89" t="s">
         <v>244</v>
       </c>
-      <c r="B55" s="99"/>
-      <c r="C55" s="99"/>
-      <c r="D55" s="99"/>
-      <c r="E55" s="99"/>
-      <c r="F55" s="99"/>
-      <c r="G55" s="99"/>
-      <c r="H55" s="99"/>
-      <c r="I55" s="99"/>
-      <c r="J55" s="100"/>
+      <c r="B55" s="90"/>
+      <c r="C55" s="90"/>
+      <c r="D55" s="90"/>
+      <c r="E55" s="90"/>
+      <c r="F55" s="90"/>
+      <c r="G55" s="90"/>
+      <c r="H55" s="90"/>
+      <c r="I55" s="90"/>
+      <c r="J55" s="91"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="25">
@@ -6535,18 +6556,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A66" s="98" t="s">
+      <c r="A66" s="89" t="s">
         <v>246</v>
       </c>
-      <c r="B66" s="99"/>
-      <c r="C66" s="99"/>
-      <c r="D66" s="99"/>
-      <c r="E66" s="99"/>
-      <c r="F66" s="99"/>
-      <c r="G66" s="99"/>
-      <c r="H66" s="99"/>
-      <c r="I66" s="99"/>
-      <c r="J66" s="100"/>
+      <c r="B66" s="90"/>
+      <c r="C66" s="90"/>
+      <c r="D66" s="90"/>
+      <c r="E66" s="90"/>
+      <c r="F66" s="90"/>
+      <c r="G66" s="90"/>
+      <c r="H66" s="90"/>
+      <c r="I66" s="90"/>
+      <c r="J66" s="91"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="25">
@@ -6901,18 +6922,18 @@
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A78" s="98" t="s">
+      <c r="A78" s="89" t="s">
         <v>345</v>
       </c>
-      <c r="B78" s="99"/>
-      <c r="C78" s="99"/>
-      <c r="D78" s="99"/>
-      <c r="E78" s="99"/>
-      <c r="F78" s="99"/>
-      <c r="G78" s="99"/>
-      <c r="H78" s="99"/>
-      <c r="I78" s="99"/>
-      <c r="J78" s="100"/>
+      <c r="B78" s="90"/>
+      <c r="C78" s="90"/>
+      <c r="D78" s="90"/>
+      <c r="E78" s="90"/>
+      <c r="F78" s="90"/>
+      <c r="G78" s="90"/>
+      <c r="H78" s="90"/>
+      <c r="I78" s="90"/>
+      <c r="J78" s="91"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="25">
@@ -7779,18 +7800,18 @@
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A106" s="86" t="s">
+      <c r="A106" s="92" t="s">
         <v>374</v>
       </c>
-      <c r="B106" s="86"/>
-      <c r="C106" s="86"/>
-      <c r="D106" s="86"/>
-      <c r="E106" s="86"/>
-      <c r="F106" s="86"/>
-      <c r="G106" s="86"/>
-      <c r="H106" s="86"/>
-      <c r="I106" s="86"/>
-      <c r="J106" s="86"/>
+      <c r="B106" s="92"/>
+      <c r="C106" s="92"/>
+      <c r="D106" s="92"/>
+      <c r="E106" s="92"/>
+      <c r="F106" s="92"/>
+      <c r="G106" s="92"/>
+      <c r="H106" s="92"/>
+      <c r="I106" s="92"/>
+      <c r="J106" s="92"/>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="25">
@@ -8283,18 +8304,18 @@
       <c r="X120" s="52"/>
     </row>
     <row r="121" spans="1:24" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A121" s="87" t="s">
+      <c r="A121" s="93" t="s">
         <v>376</v>
       </c>
-      <c r="B121" s="87"/>
-      <c r="C121" s="87"/>
-      <c r="D121" s="87"/>
-      <c r="E121" s="87"/>
-      <c r="F121" s="87"/>
-      <c r="G121" s="87"/>
-      <c r="H121" s="87"/>
-      <c r="I121" s="87"/>
-      <c r="J121" s="87"/>
+      <c r="B121" s="93"/>
+      <c r="C121" s="93"/>
+      <c r="D121" s="93"/>
+      <c r="E121" s="93"/>
+      <c r="F121" s="93"/>
+      <c r="G121" s="93"/>
+      <c r="H121" s="93"/>
+      <c r="I121" s="93"/>
+      <c r="J121" s="93"/>
       <c r="K121" s="51"/>
       <c r="L121" s="52"/>
       <c r="M121" s="52"/>
@@ -8357,18 +8378,18 @@
       <c r="X122" s="52"/>
     </row>
     <row r="123" spans="1:24" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A123" s="87" t="s">
+      <c r="A123" s="93" t="s">
         <v>381</v>
       </c>
-      <c r="B123" s="87"/>
-      <c r="C123" s="87"/>
-      <c r="D123" s="87"/>
-      <c r="E123" s="87"/>
-      <c r="F123" s="87"/>
-      <c r="G123" s="87"/>
-      <c r="H123" s="87"/>
-      <c r="I123" s="87"/>
-      <c r="J123" s="87"/>
+      <c r="B123" s="93"/>
+      <c r="C123" s="93"/>
+      <c r="D123" s="93"/>
+      <c r="E123" s="93"/>
+      <c r="F123" s="93"/>
+      <c r="G123" s="93"/>
+      <c r="H123" s="93"/>
+      <c r="I123" s="93"/>
+      <c r="J123" s="93"/>
       <c r="K123" s="51"/>
       <c r="L123" s="52"/>
       <c r="M123" s="52"/>
@@ -8431,18 +8452,18 @@
       <c r="X124" s="52"/>
     </row>
     <row r="125" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="87" t="s">
+      <c r="A125" s="93" t="s">
         <v>394</v>
       </c>
-      <c r="B125" s="87"/>
-      <c r="C125" s="87"/>
-      <c r="D125" s="87"/>
-      <c r="E125" s="87"/>
-      <c r="F125" s="87"/>
-      <c r="G125" s="87"/>
-      <c r="H125" s="87"/>
-      <c r="I125" s="87"/>
-      <c r="J125" s="87"/>
+      <c r="B125" s="93"/>
+      <c r="C125" s="93"/>
+      <c r="D125" s="93"/>
+      <c r="E125" s="93"/>
+      <c r="F125" s="93"/>
+      <c r="G125" s="93"/>
+      <c r="H125" s="93"/>
+      <c r="I125" s="93"/>
+      <c r="J125" s="93"/>
     </row>
     <row r="126" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A126" s="25">
@@ -8767,18 +8788,18 @@
       <c r="X132" s="52"/>
     </row>
     <row r="133" spans="1:24" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A133" s="87" t="s">
+      <c r="A133" s="93" t="s">
         <v>411</v>
       </c>
-      <c r="B133" s="87"/>
-      <c r="C133" s="87"/>
-      <c r="D133" s="88"/>
-      <c r="E133" s="88"/>
-      <c r="F133" s="88"/>
-      <c r="G133" s="88"/>
-      <c r="H133" s="88"/>
-      <c r="I133" s="88"/>
-      <c r="J133" s="88"/>
+      <c r="B133" s="93"/>
+      <c r="C133" s="93"/>
+      <c r="D133" s="94"/>
+      <c r="E133" s="94"/>
+      <c r="F133" s="94"/>
+      <c r="G133" s="94"/>
+      <c r="H133" s="94"/>
+      <c r="I133" s="94"/>
+      <c r="J133" s="94"/>
       <c r="K133" s="52"/>
       <c r="L133" s="52"/>
       <c r="M133" s="52"/>
@@ -9273,18 +9294,18 @@
       <c r="X144" s="52"/>
     </row>
     <row r="145" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A145" s="92" t="s">
+      <c r="A145" s="98" t="s">
         <v>439</v>
       </c>
-      <c r="B145" s="93"/>
-      <c r="C145" s="93"/>
-      <c r="D145" s="93"/>
-      <c r="E145" s="93"/>
-      <c r="F145" s="93"/>
-      <c r="G145" s="93"/>
-      <c r="H145" s="93"/>
-      <c r="I145" s="93"/>
-      <c r="J145" s="94"/>
+      <c r="B145" s="99"/>
+      <c r="C145" s="99"/>
+      <c r="D145" s="99"/>
+      <c r="E145" s="99"/>
+      <c r="F145" s="99"/>
+      <c r="G145" s="99"/>
+      <c r="H145" s="99"/>
+      <c r="I145" s="99"/>
+      <c r="J145" s="100"/>
       <c r="K145" s="52"/>
       <c r="L145" s="52"/>
       <c r="M145" s="52"/>
@@ -9731,18 +9752,18 @@
       <c r="Z155" s="52"/>
     </row>
     <row r="156" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A156" s="87" t="s">
+      <c r="A156" s="93" t="s">
         <v>510</v>
       </c>
-      <c r="B156" s="87"/>
-      <c r="C156" s="87"/>
-      <c r="D156" s="87"/>
-      <c r="E156" s="87"/>
-      <c r="F156" s="87"/>
-      <c r="G156" s="87"/>
-      <c r="H156" s="87"/>
-      <c r="I156" s="87"/>
-      <c r="J156" s="87"/>
+      <c r="B156" s="93"/>
+      <c r="C156" s="93"/>
+      <c r="D156" s="93"/>
+      <c r="E156" s="93"/>
+      <c r="F156" s="93"/>
+      <c r="G156" s="93"/>
+      <c r="H156" s="93"/>
+      <c r="I156" s="93"/>
+      <c r="J156" s="93"/>
       <c r="K156" s="52"/>
       <c r="L156" s="52"/>
       <c r="M156" s="52"/>
@@ -9809,18 +9830,18 @@
       <c r="Z157" s="52"/>
     </row>
     <row r="158" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A158" s="87" t="s">
+      <c r="A158" s="93" t="s">
         <v>536</v>
       </c>
-      <c r="B158" s="87"/>
-      <c r="C158" s="87"/>
-      <c r="D158" s="87"/>
-      <c r="E158" s="87"/>
-      <c r="F158" s="87"/>
-      <c r="G158" s="87"/>
-      <c r="H158" s="87"/>
-      <c r="I158" s="87"/>
-      <c r="J158" s="87"/>
+      <c r="B158" s="93"/>
+      <c r="C158" s="93"/>
+      <c r="D158" s="93"/>
+      <c r="E158" s="93"/>
+      <c r="F158" s="93"/>
+      <c r="G158" s="93"/>
+      <c r="H158" s="93"/>
+      <c r="I158" s="93"/>
+      <c r="J158" s="93"/>
       <c r="K158" s="52"/>
       <c r="L158" s="52"/>
       <c r="M158" s="52"/>
@@ -10655,18 +10676,18 @@
       </c>
     </row>
     <row r="180" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A180" s="87" t="s">
+      <c r="A180" s="93" t="s">
         <v>707</v>
       </c>
-      <c r="B180" s="87"/>
-      <c r="C180" s="87"/>
+      <c r="B180" s="93"/>
+      <c r="C180" s="93"/>
       <c r="D180" s="85"/>
-      <c r="E180" s="87"/>
-      <c r="F180" s="87"/>
-      <c r="G180" s="87"/>
-      <c r="H180" s="87"/>
-      <c r="I180" s="87"/>
-      <c r="J180" s="87"/>
+      <c r="E180" s="93"/>
+      <c r="F180" s="93"/>
+      <c r="G180" s="93"/>
+      <c r="H180" s="93"/>
+      <c r="I180" s="93"/>
+      <c r="J180" s="93"/>
     </row>
     <row r="181" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A181" s="62">
@@ -10957,18 +10978,18 @@
       </c>
     </row>
     <row r="190" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A190" s="89" t="s">
+      <c r="A190" s="95" t="s">
         <v>609</v>
       </c>
-      <c r="B190" s="90"/>
-      <c r="C190" s="90"/>
-      <c r="D190" s="90"/>
-      <c r="E190" s="90"/>
-      <c r="F190" s="90"/>
-      <c r="G190" s="90"/>
-      <c r="H190" s="90"/>
-      <c r="I190" s="90"/>
-      <c r="J190" s="91"/>
+      <c r="B190" s="96"/>
+      <c r="C190" s="96"/>
+      <c r="D190" s="96"/>
+      <c r="E190" s="96"/>
+      <c r="F190" s="96"/>
+      <c r="G190" s="96"/>
+      <c r="H190" s="96"/>
+      <c r="I190" s="96"/>
+      <c r="J190" s="97"/>
     </row>
     <row r="191" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A191" s="62">
@@ -13810,25 +13831,87 @@
         <v>13</v>
       </c>
     </row>
+    <row r="291" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A291" s="85" t="s">
+        <v>993</v>
+      </c>
+      <c r="B291" s="85"/>
+      <c r="C291" s="85"/>
+      <c r="D291" s="85"/>
+      <c r="E291" s="85"/>
+      <c r="F291" s="85"/>
+      <c r="G291" s="85"/>
+      <c r="H291" s="85"/>
+      <c r="I291" s="85"/>
+      <c r="J291" s="85"/>
+    </row>
+    <row r="292" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A292">
+        <v>1</v>
+      </c>
+      <c r="B292" t="s">
+        <v>10</v>
+      </c>
+      <c r="C292" t="s">
+        <v>994</v>
+      </c>
+      <c r="D292" t="s">
+        <v>995</v>
+      </c>
+      <c r="E292" t="s">
+        <v>14</v>
+      </c>
+      <c r="F292" t="s">
+        <v>996</v>
+      </c>
+      <c r="G292" t="s">
+        <v>11</v>
+      </c>
+      <c r="H292" t="s">
+        <v>970</v>
+      </c>
+      <c r="I292" t="s">
+        <v>12</v>
+      </c>
+      <c r="J292" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="293" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A293">
+        <v>2</v>
+      </c>
+      <c r="B293" t="s">
+        <v>10</v>
+      </c>
+      <c r="C293" t="s">
+        <v>997</v>
+      </c>
+      <c r="D293" t="s">
+        <v>998</v>
+      </c>
+      <c r="E293" t="s">
+        <v>14</v>
+      </c>
+      <c r="F293" t="s">
+        <v>999</v>
+      </c>
+      <c r="G293" t="s">
+        <v>11</v>
+      </c>
+      <c r="H293" t="s">
+        <v>970</v>
+      </c>
+      <c r="I293" t="s">
+        <v>12</v>
+      </c>
+      <c r="J293" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="A205:J205"/>
-    <mergeCell ref="A226:J226"/>
-    <mergeCell ref="A259:J259"/>
-    <mergeCell ref="A256:J256"/>
-    <mergeCell ref="A240:J240"/>
-    <mergeCell ref="A238:J238"/>
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="A66:J66"/>
-    <mergeCell ref="A78:J78"/>
-    <mergeCell ref="A267:J267"/>
-    <mergeCell ref="A281:J281"/>
-    <mergeCell ref="A279:J279"/>
-    <mergeCell ref="A265:J265"/>
-    <mergeCell ref="A220:J220"/>
-    <mergeCell ref="A276:J276"/>
+  <mergeCells count="34">
+    <mergeCell ref="A291:J291"/>
     <mergeCell ref="A289:J289"/>
     <mergeCell ref="A286:J286"/>
     <mergeCell ref="A273:J273"/>
@@ -13845,6 +13928,23 @@
     <mergeCell ref="A156:J156"/>
     <mergeCell ref="A158:J158"/>
     <mergeCell ref="A180:J180"/>
+    <mergeCell ref="A267:J267"/>
+    <mergeCell ref="A281:J281"/>
+    <mergeCell ref="A279:J279"/>
+    <mergeCell ref="A265:J265"/>
+    <mergeCell ref="A220:J220"/>
+    <mergeCell ref="A276:J276"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A37:J37"/>
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="A66:J66"/>
+    <mergeCell ref="A78:J78"/>
+    <mergeCell ref="A205:J205"/>
+    <mergeCell ref="A226:J226"/>
+    <mergeCell ref="A259:J259"/>
+    <mergeCell ref="A256:J256"/>
+    <mergeCell ref="A240:J240"/>
+    <mergeCell ref="A238:J238"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <conditionalFormatting sqref="E2:J2 E8:J21 E23:J23">
@@ -13942,7 +14042,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE74813B-34A6-48F5-8B35-1C10409ED694}">
-  <dimension ref="A1:AG265"/>
+  <dimension ref="A1:AG267"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="48.88671875" customWidth="1"/>
@@ -37595,6 +37695,208 @@
         <v>22</v>
       </c>
       <c r="AG265" s="28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="266" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A266" t="s">
+        <v>996</v>
+      </c>
+      <c r="B266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="D266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="F266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="G266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="H266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="I266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="J266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="K266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="L266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="M266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="N266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="O266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="P266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="R266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="S266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="T266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="U266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="V266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="W266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="X266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AC266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AF266" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AG266" s="28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="267" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A267" t="s">
+        <v>999</v>
+      </c>
+      <c r="B267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="D267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="F267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="G267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="H267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="I267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="J267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="K267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="L267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="M267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="N267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="O267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="P267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="R267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="S267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="T267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="U267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="V267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="W267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="X267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AC267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AF267" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="AG267" s="28" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>